<commit_message>
Camara frontal para YOLO + sm_planner del proyecto final
</commit_message>
<xml_diff>
--- a/ros2_ws/resultados_astar.xlsx
+++ b/ros2_ws/resultados_astar.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -619,6 +619,46 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>(-0.00, 0.00)</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>(1.12, 2.73)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>24.19</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
sm_planner con busqueda visual + YOLO, stack proyecto final funcionando, YOLO en CPU
</commit_message>
<xml_diff>
--- a/ros2_ws/resultados_astar.xlsx
+++ b/ros2_ws/resultados_astar.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -659,6 +659,86 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>(-0.00, -0.00)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>(0.50, 3.00)</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>26.42</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>(-0.00, -0.00)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>(0.00, 3.00)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>1386.22</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Sin ruta</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
Navegacion al objeto detectado: patrulla + vision (area_rel) + a_star hacia objeto
</commit_message>
<xml_diff>
--- a/ros2_ws/resultados_astar.xlsx
+++ b/ros2_ws/resultados_astar.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -739,6 +739,1406 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>(0.01, -0.01)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>(0.50, 3.00)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>15.83</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>(0.49, 2.74)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>(0.50, 3.00)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>(-0.00, 0.00)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>(0.82, -4.30)</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>1440.94</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Sin ruta</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>(-0.00, -0.00)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>(0.17, -2.61)</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>11.46</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>(-0.03, -2.34)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>(5.76, -1.38)</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Sin ruta</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>(-0.00, -0.00)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>(1.69, -2.41)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>15.23</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>(-0.00, 0.00)</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>(1.69, -2.41)</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>16.32</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>(1.43, -2.38)</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>(5.76, -1.38)</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>33.18</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>86</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>(5.53, -1.58)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>(9.70, -1.12)</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>31.82</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>84</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>(9.51, -1.38)</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>(10.34, 3.10)</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>41.59</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>(10.15, 2.83)</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>(3.45, 2.38)</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>72.45</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>149</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>(3.72, 2.76)</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>(4.59, 5.98)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>26.82</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>(4.28, 5.94)</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>(-2.56, 1.58)</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>178.02</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>142</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>(-0.00, 0.00)</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>(2.93, -2.41)</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>36.07</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>68</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>(-0.00, -0.00)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>(2.93, -2.41)</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>36.99</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>76</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>(2.66, -2.34)</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>(8.88, -1.63)</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>86.11</v>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>125</v>
+      </c>
+      <c r="I24" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>(8.70, -1.38)</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>(10.83, 2.57)</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>78.67</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>(10.63, 2.39)</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>(3.30, 2.51)</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>126.92</v>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>152</v>
+      </c>
+      <c r="I26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>(3.54, 2.50)</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>(-2.30, -1.16)</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>117</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>(-0.00, 0.00)</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>(2.93, -2.41)</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>39.14</v>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>76</v>
+      </c>
+      <c r="I28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>(3.46, -2.08)</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>(8.88, -1.63)</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>65.36</v>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>109</v>
+      </c>
+      <c r="I29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>(8.72, -1.38)</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>(10.83, 2.57)</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G30" s="3" t="n">
+        <v>46.38</v>
+      </c>
+      <c r="H30" s="3" t="n">
+        <v>79</v>
+      </c>
+      <c r="I30" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>(10.64, 2.38)</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>(3.30, 2.51)</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>172.73</v>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>152</v>
+      </c>
+      <c r="I31" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>(3.54, 2.47)</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>(-2.30, -1.16)</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>90.08</v>
+      </c>
+      <c r="H32" s="3" t="n">
+        <v>117</v>
+      </c>
+      <c r="I32" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>(-1.99, -1.15)</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>(-3.88, 1.65)</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>117.3</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>83</v>
+      </c>
+      <c r="I33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>(-0.00, 0.00)</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>(2.93, -2.41)</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F34" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G34" s="3" t="n">
+        <v>84.83</v>
+      </c>
+      <c r="H34" s="3" t="n">
+        <v>75</v>
+      </c>
+      <c r="I34" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>(2.73, -2.64)</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>(9.86, -0.21)</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>106.75</v>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>142</v>
+      </c>
+      <c r="I35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>(9.65, -0.46)</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>(8.88, -1.63)</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G36" s="3" t="n">
+        <v>7.12</v>
+      </c>
+      <c r="H36" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="I36" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>(9.02, -1.37)</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>(10.83, 2.57)</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>85.59</v>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>(-0.00, -0.00)</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>(2.93, -2.41)</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G38" s="3" t="n">
+        <v>73.13</v>
+      </c>
+      <c r="H38" s="3" t="n">
+        <v>75</v>
+      </c>
+      <c r="I38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>(2.70, -2.68)</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>(8.88, -1.63)</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F39" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G39" s="4" t="n">
+        <v>102.28</v>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>124</v>
+      </c>
+      <c r="I39" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>(8.76, -1.36)</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>(10.83, 2.57)</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F40" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>100.25</v>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>79</v>
+      </c>
+      <c r="I40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>(10.65, 2.36)</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>(3.30, 2.51)</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>130.18</v>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>154</v>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>(3.54, 2.43)</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>(-2.30, -1.16)</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F42" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>152.55</v>
+      </c>
+      <c r="H42" s="3" t="n">
+        <v>117</v>
+      </c>
+      <c r="I42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>(-2.04, -1.20)</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>(-3.48, -1.84)</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>11.36</v>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>Exito</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>

</xml_diff>